<commit_message>
feat: S1/S2 missing-node gameplay (4 floating nodes, S2 patch gaps)
S1 leaves 4 unresolved nodes (leaf / stem / fruit / root) that glow red and
float out of the matrix. S2 starts with those slots empty; the player matches
details and drags each node into the right gap (auto-snap, wrong slot rejects).
All 4 patched: watering animation, then the original S2 follow-up.

Adds MissingNodePicker, alias pick spheres, halo-at / link growth, S2_NOPATH /
WRONG / PATCHED dialogue, PrimeTween 1.5.0. Main.unity is rebuilt in the next commit.
</commit_message>
<xml_diff>
--- a/docs/script/05_audio_list.xlsx
+++ b/docs/script/05_audio_list.xlsx
@@ -597,6 +597,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -611,7 +612,7 @@
         </is>
       </c>
       <c r="B5" s="4">
-        <f>COUNTA('配音'!A2:A71)</f>
+        <f>COUNTA('配音'!A2:A78)</f>
         <v/>
       </c>
     </row>
@@ -622,7 +623,7 @@
         </is>
       </c>
       <c r="B6" s="4">
-        <f>COUNTIF('配音'!G2:G71,"是")</f>
+        <f>COUNTIF('配音'!G2:G78,"是")</f>
         <v/>
       </c>
     </row>
@@ -633,7 +634,7 @@
         </is>
       </c>
       <c r="B7" s="4">
-        <f>COUNTIFS('配音'!C2:C71,"亲切的声音",'配音'!G2:G71,"是")</f>
+        <f>COUNTIFS('配音'!C2:C78,"亲切的声音",'配音'!G2:G78,"是")</f>
         <v/>
       </c>
     </row>
@@ -644,7 +645,7 @@
         </is>
       </c>
       <c r="B8" s="4">
-        <f>COUNTIFS('配音'!C2:C71,"没有温度的声音",'配音'!G2:G71,"是")</f>
+        <f>COUNTIFS('配音'!C2:C78,"没有温度的声音",'配音'!G2:G78,"是")</f>
         <v/>
       </c>
     </row>
@@ -655,7 +656,7 @@
         </is>
       </c>
       <c r="B9" s="4">
-        <f>SUMIF('配音'!G2:G71,"是",'配音'!J2:J71)</f>
+        <f>SUMIF('配音'!G2:G78,"是",'配音'!J2:J78)</f>
         <v/>
       </c>
     </row>
@@ -736,6 +737,7 @@
         <v/>
       </c>
     </row>
+    <row r="17"/>
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
         <is>
@@ -890,7 +892,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M71"/>
+  <dimension ref="A1:M78"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -4233,6 +4235,356 @@
       </c>
       <c r="J71" s="22">
         <f>ROUND(I71/$M$3+0.4,1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="21" t="inlineStr">
+        <is>
+          <t>VO_OUTRO_001</t>
+        </is>
+      </c>
+      <c r="B72" s="21" t="inlineStr">
+        <is>
+          <t>OUTRO</t>
+        </is>
+      </c>
+      <c r="C72" s="21" t="inlineStr">
+        <is>
+          <t>机械音</t>
+        </is>
+      </c>
+      <c r="D72" s="21" t="inlineStr">
+        <is>
+          <t>字幕</t>
+        </is>
+      </c>
+      <c r="E72" s="21" t="inlineStr">
+        <is>
+          <t>Neural activity signals have returned to normal levels.</t>
+        </is>
+      </c>
+      <c r="F72" s="21" t="inlineStr">
+        <is>
+          <t>治疗仓的提示音，冷静、无情绪；不同于 Agent，是医疗设备</t>
+        </is>
+      </c>
+      <c r="G72" s="21" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="H72" s="21" t="inlineStr">
+        <is>
+          <t>Outro 视频内对白，全部走字幕。原文：神经活跃信号恢复正常指标。</t>
+        </is>
+      </c>
+      <c r="I72" s="22">
+        <f>LEN(TRIM(E72))-LEN(SUBSTITUTE(E72," ",""))+1</f>
+        <v/>
+      </c>
+      <c r="J72" s="22">
+        <f>ROUND(I72/2.5+0.4,1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="21" t="inlineStr">
+        <is>
+          <t>VO_OUTRO_002</t>
+        </is>
+      </c>
+      <c r="B73" s="21" t="inlineStr">
+        <is>
+          <t>OUTRO</t>
+        </is>
+      </c>
+      <c r="C73" s="21" t="inlineStr">
+        <is>
+          <t>母亲（女声）</t>
+        </is>
+      </c>
+      <c r="D73" s="21" t="inlineStr">
+        <is>
+          <t>字幕</t>
+        </is>
+      </c>
+      <c r="E73" s="21" t="inlineStr">
+        <is>
+          <t>Did she just blink?</t>
+        </is>
+      </c>
+      <c r="F73" s="21" t="inlineStr">
+        <is>
+          <t>紧张、不敢相信，压低声音</t>
+        </is>
+      </c>
+      <c r="G73" s="21" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="H73" s="21" t="inlineStr">
+        <is>
+          <t>Outro 视频内对白，全部走字幕。原文：眨眼了？</t>
+        </is>
+      </c>
+      <c r="I73" s="22">
+        <f>LEN(TRIM(E73))-LEN(SUBSTITUTE(E73," ",""))+1</f>
+        <v/>
+      </c>
+      <c r="J73" s="22">
+        <f>ROUND(I73/2.5+0.4,1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="21" t="inlineStr">
+        <is>
+          <t>VO_OUTRO_003</t>
+        </is>
+      </c>
+      <c r="B74" s="21" t="inlineStr">
+        <is>
+          <t>OUTRO</t>
+        </is>
+      </c>
+      <c r="C74" s="21" t="inlineStr">
+        <is>
+          <t>医生（男声）</t>
+        </is>
+      </c>
+      <c r="D74" s="21" t="inlineStr">
+        <is>
+          <t>字幕</t>
+        </is>
+      </c>
+      <c r="E74" s="21" t="inlineStr">
+        <is>
+          <t>She's awake!</t>
+        </is>
+      </c>
+      <c r="F74" s="21" t="inlineStr">
+        <is>
+          <t>惊喜，脱口而出</t>
+        </is>
+      </c>
+      <c r="G74" s="21" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="H74" s="21" t="inlineStr">
+        <is>
+          <t>Outro 视频内对白，全部走字幕。原文：醒了！</t>
+        </is>
+      </c>
+      <c r="I74" s="22">
+        <f>LEN(TRIM(E74))-LEN(SUBSTITUTE(E74," ",""))+1</f>
+        <v/>
+      </c>
+      <c r="J74" s="22">
+        <f>ROUND(I74/2.5+0.4,1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="21" t="inlineStr">
+        <is>
+          <t>VO_OUTRO_004</t>
+        </is>
+      </c>
+      <c r="B75" s="21" t="inlineStr">
+        <is>
+          <t>OUTRO</t>
+        </is>
+      </c>
+      <c r="C75" s="21" t="inlineStr">
+        <is>
+          <t>医生（女声）</t>
+        </is>
+      </c>
+      <c r="D75" s="21" t="inlineStr">
+        <is>
+          <t>字幕</t>
+        </is>
+      </c>
+      <c r="E75" s="21" t="inlineStr">
+        <is>
+          <t>Yes, she's awake.</t>
+        </is>
+      </c>
+      <c r="F75" s="21" t="inlineStr">
+        <is>
+          <t>平稳确认，带一点欣慰</t>
+        </is>
+      </c>
+      <c r="G75" s="21" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="H75" s="21" t="inlineStr">
+        <is>
+          <t>Outro 视频内对白，全部走字幕。原文：是的，她醒了。</t>
+        </is>
+      </c>
+      <c r="I75" s="22">
+        <f>LEN(TRIM(E75))-LEN(SUBSTITUTE(E75," ",""))+1</f>
+        <v/>
+      </c>
+      <c r="J75" s="22">
+        <f>ROUND(I75/2.5+0.4,1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="21" t="inlineStr">
+        <is>
+          <t>VO_OUTRO_005</t>
+        </is>
+      </c>
+      <c r="B76" s="21" t="inlineStr">
+        <is>
+          <t>OUTRO</t>
+        </is>
+      </c>
+      <c r="C76" s="21" t="inlineStr">
+        <is>
+          <t>亲切的声音</t>
+        </is>
+      </c>
+      <c r="D76" s="21" t="inlineStr">
+        <is>
+          <t>字幕</t>
+        </is>
+      </c>
+      <c r="E76" s="21" t="inlineStr">
+        <is>
+          <t>Hey, lucky one. For a patient with severe Cognitive Impoverishment Syndrome, to complete your perceptual recovery by following the guidance in such a short time... that's truly remarkable.</t>
+        </is>
+      </c>
+      <c r="F76" s="21" t="inlineStr">
+        <is>
+          <t>治疗师背对画面，越肩镜头；就是游戏里一直引导你的那个温柔女声，现在第一次以真人出现</t>
+        </is>
+      </c>
+      <c r="G76" s="21" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="H76" s="21" t="inlineStr">
+        <is>
+          <t>Outro 视频内对白，全部走字幕。原文：嗨，幸运儿。作为一个认知贫化症重度患者，在这么短的时间内就成功跟随指引完成了感知恢复，真是令人惊讶。</t>
+        </is>
+      </c>
+      <c r="I76" s="22">
+        <f>LEN(TRIM(E76))-LEN(SUBSTITUTE(E76," ",""))+1</f>
+        <v/>
+      </c>
+      <c r="J76" s="22">
+        <f>ROUND(I76/2.5+0.4,1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="21" t="inlineStr">
+        <is>
+          <t>VO_OUTRO_006</t>
+        </is>
+      </c>
+      <c r="B77" s="21" t="inlineStr">
+        <is>
+          <t>OUTRO</t>
+        </is>
+      </c>
+      <c r="C77" s="21" t="inlineStr">
+        <is>
+          <t>亲切的声音</t>
+        </is>
+      </c>
+      <c r="D77" s="21" t="inlineStr">
+        <is>
+          <t>字幕</t>
+        </is>
+      </c>
+      <c r="E77" s="21" t="inlineStr">
+        <is>
+          <t>Looks like the gift your mother brought really did reach your soul. Your ghost.</t>
+        </is>
+      </c>
+      <c r="F77" s="21" t="inlineStr">
+        <is>
+          <t>镜头切到窗台的番茄；温柔，带笑意，ghost 点题</t>
+        </is>
+      </c>
+      <c r="G77" s="21" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="H77" s="21" t="inlineStr">
+        <is>
+          <t>Outro 视频内对白，全部走字幕。原文：看来你母亲带来的这份礼物，确实到达了你的灵魂（ghost）。</t>
+        </is>
+      </c>
+      <c r="I77" s="22">
+        <f>LEN(TRIM(E77))-LEN(SUBSTITUTE(E77," ",""))+1</f>
+        <v/>
+      </c>
+      <c r="J77" s="22">
+        <f>ROUND(I77/2.5+0.4,1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="21" t="inlineStr">
+        <is>
+          <t>VO_OUTRO_007</t>
+        </is>
+      </c>
+      <c r="B78" s="21" t="inlineStr">
+        <is>
+          <t>OUTRO</t>
+        </is>
+      </c>
+      <c r="C78" s="21" t="inlineStr">
+        <is>
+          <t>母亲（女声）</t>
+        </is>
+      </c>
+      <c r="D78" s="21" t="inlineStr">
+        <is>
+          <t>字幕</t>
+        </is>
+      </c>
+      <c r="E78" s="21" t="inlineStr">
+        <is>
+          <t>Welcome back.</t>
+        </is>
+      </c>
+      <c r="F78" s="21" t="inlineStr">
+        <is>
+          <t>从窗外越过番茄往里看，母亲抱住女儿；哽咽、很轻，全片最后一句</t>
+        </is>
+      </c>
+      <c r="G78" s="21" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="H78" s="21" t="inlineStr">
+        <is>
+          <t>Outro 视频内对白，全部走字幕。原文：欢迎回来。</t>
+        </is>
+      </c>
+      <c r="I78" s="22">
+        <f>LEN(TRIM(E78))-LEN(SUBSTITUTE(E78," ",""))+1</f>
+        <v/>
+      </c>
+      <c r="J78" s="22">
+        <f>ROUND(I78/2.5+0.4,1)</f>
         <v/>
       </c>
     </row>

</xml_diff>